<commit_message>
0.5.0: guided setup, one-command sources, demo and doctor
- unwalled setup (also "unwalled" alone in a terminal): checks the
  computer, offers to install the command, adds unwalled to Claude Code,
  Claude Desktop, Cursor, Windsurf, VS Code, Gemini CLI and Codex
  (plain JSON only, with backups; --yes, --remove), connects a first
  source or the demo
- unwalled add <source>: kind of source detected, name suggested
- unwalled demo, unwalled key (hidden input), unwalled doctor
- server instructions mention files, databases and presets
- English fixtures; tool summaries without "by order" / "a order"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventes 2026" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales 2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,22 +420,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>produit</t>
+          <t>product</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>quantité</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>prix</t>
+          <t>price</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>payé</t>
+          <t>paid</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>lampe</t>
+          <t>lamp</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -461,14 +461,14 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>rouge &amp; bleu</t>
+          <t>red &amp; blue</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chaise</t>
+          <t>chair</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -481,6 +481,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -513,9 +514,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B4"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
@@ -524,7 +526,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>nom</t>
+          <t>name</t>
         </is>
       </c>
     </row>
@@ -544,7 +546,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Globex</t>
+          <t>Zürich Café GmbH</t>
         </is>
       </c>
     </row>

</xml_diff>